<commit_message>
fix: defer DrawingsPart DOM loading to avoid re-serialization of unchanged drawings
Accessing WorksheetDrawing eagerly caused the OpenXML SDK to load the
drawing DOM for every worksheet, even when the part wouldn't be deleted.
The re-serialized DOM differed from the original XML, breaking save
comparisons for charts, form controls, and shape-containing worksheets.

Move the HasChildren check to be the last short-circuit condition so it
only evaluates when all other deletion criteria are met. Update the
WorksheetWithDrawingCanBeModified expected output to include the
preserved shape per #2377.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/XLibur.Tests/Resource/Other/Parts/WorksheetWithDrawingCanBeModified-output.xlsx
+++ b/XLibur.Tests/Resource/Other/Parts/WorksheetWithDrawingCanBeModified-output.xlsx
@@ -101,6 +101,71 @@
     </x:ext>
   </x:extLst>
 </x:styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>285750</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>57150</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>190500</xdr:colOff>
+      <xdr:row>6</xdr:row>
+      <xdr:rowOff>66675</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="2" name="Rectangle 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{2CBB2917-8659-40E1-73F8-620F66A9D93B}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="285750" y="628650"/>
+          <a:ext cx="1733550" cy="581025"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1">
+            <a:shade val="15000"/>
+          </a:schemeClr>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:endParaRPr lang="en-US" sz="1100"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -416,6 +481,7 @@
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:pageSetup paperSize="1" scale="100" pageOrder="downThenOver" orientation="default" blackAndWhite="0" draft="0" cellComments="none" errors="displayed"/>
   <x:headerFooter/>
+  <x:drawing r:id="rId1"/>
   <x:tableParts count="0"/>
 </x:worksheet>
 </file>
</xml_diff>